<commit_message>
Initial commit: Capstone project deliverables
</commit_message>
<xml_diff>
--- a/HealthFirst_Data_Analysis.xlsx
+++ b/HealthFirst_Data_Analysis.xlsx
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>91</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -544,11 +544,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9">
@@ -559,11 +559,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10">
@@ -574,11 +574,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>92</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>38</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12">
@@ -604,11 +604,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>73</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14">
@@ -634,11 +634,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15">
@@ -649,11 +649,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -664,11 +664,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>83</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -679,11 +679,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -694,11 +694,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>89</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19">
@@ -709,11 +709,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20">
@@ -724,11 +724,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21">
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>28</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22">
@@ -754,11 +754,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>66</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23">
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>90</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24">
@@ -784,11 +784,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>118</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>5</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26">
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>76</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27">
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28">
@@ -844,11 +844,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>22</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29">
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>102</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>94</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31">
@@ -889,11 +889,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>114</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>58</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33">
@@ -919,11 +919,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>32</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34">
@@ -934,11 +934,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>118</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35">
@@ -949,11 +949,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36">
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37">
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>31</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38">
@@ -994,11 +994,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39">
@@ -1009,11 +1009,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40">
@@ -1024,11 +1024,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
@@ -1039,11 +1039,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42">
@@ -1054,11 +1054,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="43">
@@ -1069,11 +1069,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>17</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44">
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>102</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>78</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
@@ -1114,11 +1114,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>96</v>
+        <v>118</v>
       </c>
     </row>
     <row r="47">
@@ -1129,11 +1129,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>12</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48">
@@ -1144,11 +1144,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>92</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49">
@@ -1163,7 +1163,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>118</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50">
@@ -1174,11 +1174,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51">
@@ -1189,11 +1189,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>93</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52">
@@ -1204,11 +1204,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>11</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53">
@@ -1219,11 +1219,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>100</v>
+        <v>7</v>
       </c>
     </row>
     <row r="54">
@@ -1234,11 +1234,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="55">
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>7</v>
+        <v>61</v>
       </c>
     </row>
     <row r="56">
@@ -1264,11 +1264,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="57">
@@ -1279,11 +1279,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>92</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58">
@@ -1294,11 +1294,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
     </row>
     <row r="59">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>54</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60">
@@ -1324,11 +1324,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>23</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61">
@@ -1339,11 +1339,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="62">
@@ -1354,11 +1354,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>62</v>
+        <v>35</v>
       </c>
     </row>
     <row r="63">
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>13</v>
+        <v>108</v>
       </c>
     </row>
     <row r="64">
@@ -1388,7 +1388,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>26</v>
+        <v>84</v>
       </c>
     </row>
     <row r="65">
@@ -1399,11 +1399,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>34</v>
+        <v>106</v>
       </c>
     </row>
     <row r="66">
@@ -1414,11 +1414,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>28</v>
+        <v>102</v>
       </c>
     </row>
     <row r="67">
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="68">
@@ -1444,11 +1444,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>52</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69">
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
     </row>
     <row r="70">
@@ -1474,11 +1474,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>63</v>
+        <v>25</v>
       </c>
     </row>
     <row r="71">
@@ -1489,11 +1489,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="72">
@@ -1504,11 +1504,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="73">
@@ -1519,11 +1519,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>95</v>
+        <v>27</v>
       </c>
     </row>
     <row r="74">
@@ -1538,7 +1538,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
     </row>
     <row r="75">
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>106</v>
+        <v>13</v>
       </c>
     </row>
     <row r="76">
@@ -1564,11 +1564,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>86</v>
+        <v>103</v>
       </c>
     </row>
     <row r="77">
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
     </row>
     <row r="78">
@@ -1594,11 +1594,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="79">
@@ -1609,11 +1609,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="80">
@@ -1624,11 +1624,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="81">
@@ -1639,11 +1639,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>98</v>
+        <v>15</v>
       </c>
     </row>
     <row r="82">
@@ -1654,11 +1654,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>13</v>
+        <v>87</v>
       </c>
     </row>
     <row r="83">
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="84">
@@ -1684,11 +1684,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>32</v>
+        <v>65</v>
       </c>
     </row>
     <row r="85">
@@ -1699,11 +1699,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>53</v>
+        <v>19</v>
       </c>
     </row>
     <row r="86">
@@ -1714,11 +1714,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
     </row>
     <row r="87">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>53</v>
+        <v>11</v>
       </c>
     </row>
     <row r="88">
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>67</v>
+        <v>16</v>
       </c>
     </row>
     <row r="89">
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>104</v>
+        <v>18</v>
       </c>
     </row>
     <row r="90">
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>106</v>
+        <v>14</v>
       </c>
     </row>
     <row r="91">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="92">
@@ -1808,7 +1808,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>102</v>
+        <v>9</v>
       </c>
     </row>
     <row r="93">
@@ -1819,11 +1819,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Radiology</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>70</v>
+        <v>21</v>
       </c>
     </row>
     <row r="94">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
     </row>
     <row r="95">
@@ -1849,11 +1849,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>57</v>
+        <v>110</v>
       </c>
     </row>
     <row r="96">
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>117</v>
+        <v>59</v>
       </c>
     </row>
     <row r="97">
@@ -1879,11 +1879,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>58</v>
+        <v>105</v>
       </c>
     </row>
     <row r="98">
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>53</v>
+        <v>31</v>
       </c>
     </row>
     <row r="99">
@@ -1909,11 +1909,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>13</v>
+        <v>61</v>
       </c>
     </row>
     <row r="100">
@@ -1928,7 +1928,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>77</v>
+        <v>13</v>
       </c>
     </row>
     <row r="101">
@@ -1939,11 +1939,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>56</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60</v>
+        <v>62.1</v>
       </c>
     </row>
     <row r="3">
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61.33333333333334</v>
+        <v>57.9</v>
       </c>
     </row>
     <row r="4">
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58.88571428571429</v>
+        <v>62.66666666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>